<commit_message>
Built site for kwb.impetus: 0.0.0.9000@6395f4f
</commit_message>
<xml_diff>
--- a/impetus_flows_v1.0.0.xlsx
+++ b/impetus_flows_v1.0.0.xlsx
@@ -685,7 +685,7 @@
         <v>22</v>
       </c>
       <c r="B4" t="n">
-        <v>50338143.9273162</v>
+        <v>50338558.0632052</v>
       </c>
     </row>
     <row r="5">
@@ -693,7 +693,7 @@
         <v>23</v>
       </c>
       <c r="B5" t="n">
-        <v>39012061.54367</v>
+        <v>39012382.4989841</v>
       </c>
     </row>
     <row r="6">
@@ -701,7 +701,7 @@
         <v>24</v>
       </c>
       <c r="B6" t="n">
-        <v>31330999.0434083</v>
+        <v>31331256.806014</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Built site for kwb.impetus: 0.0.0.9000@c6931a1
</commit_message>
<xml_diff>
--- a/impetus_flows_v1.0.0.xlsx
+++ b/impetus_flows_v1.0.0.xlsx
@@ -677,7 +677,7 @@
         <v>21</v>
       </c>
       <c r="B3" t="n">
-        <v>622.41069294584</v>
+        <v>622.410692945837</v>
       </c>
     </row>
     <row r="4">
@@ -685,7 +685,7 @@
         <v>22</v>
       </c>
       <c r="B4" t="n">
-        <v>50338558.0632052</v>
+        <v>50338558.1173583</v>
       </c>
     </row>
     <row r="5">
@@ -693,7 +693,7 @@
         <v>23</v>
       </c>
       <c r="B5" t="n">
-        <v>39012382.4989841</v>
+        <v>39012382.5409527</v>
       </c>
     </row>
     <row r="6">
@@ -701,7 +701,7 @@
         <v>24</v>
       </c>
       <c r="B6" t="n">
-        <v>31331256.806014</v>
+        <v>31331256.8397193</v>
       </c>
     </row>
     <row r="7">

</xml_diff>